<commit_message>
chore: regenerate workbooks after final verification run
Byte-level only: the ENH02-TD-REG-02-01/ENH02-TD-REG-05-01 datasets embed
a timestamp-suffixed synthetic email by design, so each fresh process
regeneration naturally differs slightly -- expected, documented behavior
(see the Enhancement-02 closure report's own identical note), not new
content.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNeFKcPsJn8aSBga2ngnFw
</commit_message>
<xml_diff>
--- a/testmgmt/generated/MVP2_TestData.xlsx
+++ b/testmgmt/generated/MVP2_TestData.xlsx
@@ -6924,7 +6924,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>enh02.reg02.1789504941917@example.test</t>
+          <t>enh02.reg02.1789505041145@example.test</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -7454,7 +7454,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>enh02.shared.1789504941917@example.test</t>
+          <t>enh02.shared.1789505041145@example.test</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">

</xml_diff>